<commit_message>
feat(production): unbind replenishment slips from operations
</commit_message>
<xml_diff>
--- a/docs/samples/补料单-样例.xlsx
+++ b/docs/samples/补料单-样例.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="35">
   <si>
     <t>【补料单】</t>
   </si>
@@ -56,9 +56,6 @@
   </si>
   <si>
     <t>领料工序：</t>
-  </si>
-  <si>
-    <t>裁剪</t>
   </si>
   <si>
     <t>操作人：</t>
@@ -624,53 +621,53 @@
         <v>14</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="G7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="H7" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="E8" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="F8" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="G8" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="H8" s="4" t="s">
         <v>28</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -681,19 +678,19 @@
         <v>6</v>
       </c>
       <c r="C9" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="E9" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="F9" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="G9" s="5" t="s">
         <v>33</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>34</v>
       </c>
       <c r="H9" s="7">
         <v>12</v>
@@ -701,7 +698,7 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>

</xml_diff>